<commit_message>
SCS4 review: carry the named alternative on the two held swaps
Row 1314 (Cal King campaign) now lists Cal King White and row 871 (Twin
term on Queen Graphite) lists Twin Graphite in the Alternative child
column and the swap table, matching their reason text.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ECNUyLvUafHehET6NevFNz
</commit_message>
<xml_diff>
--- a/docs/reviews/SCS4_Review_Rows_20260924-7aed7be1.xlsx
+++ b/docs/reviews/SCS4_Review_Rows_20260924-7aed7be1.xlsx
@@ -11725,6 +11725,11 @@
       <c r="U141" t="n">
         <v>34</v>
       </c>
+      <c r="V141" t="inlineStr">
+        <is>
+          <t>SL-COOLING-SHEET-TWIN-GRAPHITE</t>
+        </is>
+      </c>
     </row>
     <row r="142">
       <c r="A142" t="n">
@@ -13851,6 +13856,11 @@
       </c>
       <c r="U167" t="n">
         <v>110</v>
+      </c>
+      <c r="V167" t="inlineStr">
+        <is>
+          <t>SL-COOLING-SHEET-CAL-KING-WHITE</t>
+        </is>
       </c>
     </row>
     <row r="168">
@@ -43690,7 +43700,11 @@
       <c r="J5" t="n">
         <v>1</v>
       </c>
-      <c r="K5" t="inlineStr"/>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>SL-COOLING-SHEET-TWIN-GRAPHITE</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -43902,7 +43916,11 @@
       <c r="J10" t="n">
         <v>1</v>
       </c>
-      <c r="K10" t="inlineStr"/>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>SL-COOLING-SHEET-CAL-KING-WHITE</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">

</xml_diff>